<commit_message>
Update credit score 2026-10-14 16:30:40
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -638,11 +638,11 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6450000</v>
+        <v>1450000</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1405/04/19 - 19:43</t>
+          <t>1405/07/22 - 16:29</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-14 17:13:51
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7216000</v>
+        <v>7266000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/19 - 18:09</t>
+          <t>1405/07/22 - 17:13</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-14 18:18:50
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2115000</v>
+        <v>2515000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/07/21 - 16:45</t>
+          <t>1405/07/22 - 18:18</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-15 16:35:25
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7266000</v>
+        <v>7366000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/22 - 17:13</t>
+          <t>1405/07/23 - 16:18</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-15 17:02:56
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7366000</v>
+        <v>7466000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/23 - 16:18</t>
+          <t>1405/07/23 - 17:02</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-16 17:00:38
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -454,11 +454,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2833000</v>
+        <v>3022000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1405/07/17 - 17:48</t>
+          <t>1405/07/24 - 16:55</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7466000</v>
+        <v>7680000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/23 - 17:02</t>
+          <t>1405/07/24 - 16:59</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2730000</v>
+        <v>2974000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/07/21 - 16:43</t>
+          <t>1405/07/24 - 16:53</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>150000</v>
+        <v>339000</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1405/06/22 - 09:58</t>
+          <t>1405/07/24 - 16:54</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -592,11 +592,11 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2363500</v>
+        <v>2552500</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1405/07/21 - 16:45</t>
+          <t>1405/07/24 - 16:57</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3282600</v>
+        <v>3471600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/07/03 - 15:20</t>
+          <t>1405/07/24 - 16:55</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-16 18:29:29
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3471600</v>
+        <v>3282600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 16:55</t>
+          <t>1405/07/24 - 18:28</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-16 18:43:30
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>87000</v>
+        <v>447000</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>1405/07/22 - 18:53</t>
+          <t>1405/07/24 - 18:42</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-16 19:01:06
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>339000</v>
+        <v>519000</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 16:54</t>
+          <t>1405/07/24 - 19:00</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-16 21:12:04
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -753,11 +753,11 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>600000</v>
+        <v>800000</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>1405/07/19 - 16:22</t>
+          <t>1405/07/24 - 21:11</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-16 21:13:21
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3282600</v>
+        <v>3342600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 18:28</t>
+          <t>1405/07/24 - 21:12</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-17 18:45:11
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2974000</v>
+        <v>2810000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 16:53</t>
+          <t>1405/07/25 - 18:42</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2515000</v>
+        <v>2705000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/07/22 - 18:18</t>
+          <t>1405/07/25 - 18:44</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-17 19:45:42
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7680000</v>
+        <v>7710000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 16:59</t>
+          <t>1405/07/25 - 19:44</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-17 20:07:17
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -454,11 +454,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3022000</v>
+        <v>2833000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 16:55</t>
+          <t>1405/07/25 - 20:06</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-18 20:46:16
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -753,11 +753,11 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>800000</v>
+        <v>927000</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 21:11</t>
+          <t>1405/07/26 - 18:51</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-19 17:23:00
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2705000</v>
+        <v>1895000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/07/25 - 18:44</t>
+          <t>1405/07/27 - 17:22</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-19 18:19:22
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>447000</v>
+        <v>1043000</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 18:42</t>
+          <t>1405/07/27 - 18:18</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-19 19:55:47
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2810000</v>
+        <v>2845000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/07/25 - 18:42</t>
+          <t>1405/07/27 - 19:54</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-20 17:27:29
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1895000</v>
+        <v>2651000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/07/27 - 17:22</t>
+          <t>1405/07/28 - 17:26</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-20 20:24:38
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3342600</v>
+        <v>3492600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 21:12</t>
+          <t>1405/07/28 - 20:23</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-21 18:23:03
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -454,11 +454,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2833000</v>
+        <v>3103000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1405/07/25 - 20:06</t>
+          <t>1405/07/29 - 18:19</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7710000</v>
+        <v>8030000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/25 - 19:44</t>
+          <t>1405/07/29 - 18:19</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2845000</v>
+        <v>3115000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/07/27 - 19:54</t>
+          <t>1405/07/29 - 18:18</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-21 19:18:21
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>519000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 19:00</t>
+          <t>1405/07/29 - 19:17</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-21 19:37:50
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -523,11 +523,11 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-9000</v>
+        <v>-549000</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1405/07/17 - 17:44</t>
+          <t>1405/07/29 - 19:37</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-22 14:58:24
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>8030000</v>
+        <v>5030000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/29 - 18:19</t>
+          <t>1405/07/30 - 14:57</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -753,11 +753,11 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>927000</v>
+        <v>-3000</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>1405/07/26 - 18:51</t>
+          <t>1405/07/30 - 14:57</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-22 20:43:57
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -592,11 +592,11 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2552500</v>
+        <v>2702500</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1405/07/24 - 16:57</t>
+          <t>1405/07/30 - 20:43</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-22 21:06:23
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -454,11 +454,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3103000</v>
+        <v>2103000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1405/07/29 - 18:19</t>
+          <t>1405/07/30 - 21:05</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-23 16:23:33
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1043000</v>
+        <v>1673000</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>1405/07/27 - 18:18</t>
+          <t>1405/08/01 - 16:22</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-23 17:49:59
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3115000</v>
+        <v>3205000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/07/29 - 18:18</t>
+          <t>1405/08/01 - 17:49</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-23 18:34:48
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2651000</v>
+        <v>2841000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/07/28 - 17:26</t>
+          <t>1405/08/01 - 18:33</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-24 20:03:28
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2841000</v>
+        <v>3056000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/08/01 - 18:33</t>
+          <t>1405/08/02 - 19:00</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-25 18:38:20
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3056000</v>
+        <v>3151000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/08/02 - 19:00</t>
+          <t>1405/08/03 - 18:37</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-26 18:04:17
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1673000</v>
+        <v>2427000</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>1405/08/01 - 16:22</t>
+          <t>1405/08/04 - 18:03</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-26 18:45:21
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3151000</v>
+        <v>3916000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/08/03 - 18:37</t>
+          <t>1405/08/04 - 18:44</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-27 18:44:20
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -592,11 +592,11 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2702500</v>
+        <v>1202500</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1405/07/30 - 20:43</t>
+          <t>1405/08/05 - 18:43</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-27 19:09:38
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5030000</v>
+        <v>5100000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/07/30 - 14:57</t>
+          <t>1405/08/05 - 19:08</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -523,11 +523,11 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-549000</v>
+        <v>-184000</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1405/07/29 - 19:37</t>
+          <t>1405/08/05 - 19:08</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-27 19:13:34
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -454,11 +454,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2103000</v>
+        <v>2238000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1405/07/30 - 21:05</t>
+          <t>1405/08/05 - 19:12</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5100000</v>
+        <v>5235000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/08/05 - 19:08</t>
+          <t>1405/08/05 - 19:12</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3205000</v>
+        <v>3250000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/08/01 - 17:49</t>
+          <t>1405/08/05 - 19:11</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-27 19:23:03
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5235000</v>
+        <v>5165000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/08/05 - 19:12</t>
+          <t>1405/08/05 - 19:22</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-28 19:59:21
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3916000</v>
+        <v>4106000</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1405/08/04 - 18:44</t>
+          <t>1405/08/06 - 19:58</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-29 20:54:29
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3492600</v>
+        <v>1492600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/07/28 - 20:23</t>
+          <t>1405/08/07 - 20:53</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-29 21:29:06
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -454,11 +454,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2238000</v>
+        <v>2363000</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1405/08/05 - 19:12</t>
+          <t>1405/08/07 - 21:27</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -477,11 +477,11 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5165000</v>
+        <v>5290000</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1405/08/05 - 19:22</t>
+          <t>1405/08/07 - 21:28</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3250000</v>
+        <v>3510000</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1405/08/05 - 19:11</t>
+          <t>1405/08/07 - 21:25</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0</v>
+        <v>125000</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1405/07/29 - 19:17</t>
+          <t>1405/08/07 - 21:26</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-30 13:36:31
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -569,11 +569,11 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3965000</v>
+        <v>4465000</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1405/07/10 - 19:20</t>
+          <t>1405/08/08 - 13:35</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1492600</v>
+        <v>1672600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/08/07 - 20:53</t>
+          <t>1405/08/08 - 13:35</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-30 18:01:28
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2427000</v>
+        <v>2922000</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>1405/08/04 - 18:03</t>
+          <t>1405/08/08 - 18:00</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-30 19:28:47
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -615,11 +615,11 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1672600</v>
+        <v>1872600</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1405/08/08 - 13:35</t>
+          <t>1405/08/08 - 19:27</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update credit score 2026-10-31 19:40:12
</commit_message>
<xml_diff>
--- a/customers.xlsx
+++ b/customers.xlsx
@@ -592,11 +592,11 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1202500</v>
+        <v>762500</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1405/08/05 - 18:43</t>
+          <t>1405/08/09 - 19:39</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">

</xml_diff>